<commit_message>
SPEC20 - Fixed code generation
</commit_message>
<xml_diff>
--- a/tests/fixtures/catalog-items-sample.xlsx
+++ b/tests/fixtures/catalog-items-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t>catalogTypeCode</t>
   </si>
@@ -19,9 +19,6 @@
     <t>catalogTypeName</t>
   </si>
   <si>
-    <t>code</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -40,82 +37,64 @@
     <t>Tipo Prueba Import</t>
   </si>
   <si>
+    <t>Activo</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Estado activo</t>
+  </si>
+  <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Cerrado</t>
+  </si>
+  <si>
+    <t>Estado cerrado</t>
+  </si>
+  <si>
+    <t>Orden</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>tipo nuevo import</t>
+  </si>
+  <si>
+    <t>Tipo Nuevo Import</t>
+  </si>
+  <si>
+    <t>Grave</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Caso grave</t>
+  </si>
+  <si>
+    <t>Leve</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>ACTIVO</t>
   </si>
   <si>
-    <t>Activo</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Estado activo</t>
-  </si>
-  <si>
-    <t>VIGENTE</t>
-  </si>
-  <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>CERRADO</t>
-  </si>
-  <si>
-    <t>Cerrado</t>
-  </si>
-  <si>
-    <t>Estado cerrado</t>
-  </si>
-  <si>
-    <t>ORDEN</t>
-  </si>
-  <si>
-    <t>Orden</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>abc</t>
-  </si>
-  <si>
-    <t>tipo nuevo import</t>
-  </si>
-  <si>
-    <t>Tipo Nuevo Import</t>
-  </si>
-  <si>
-    <t>GRAVE</t>
-  </si>
-  <si>
-    <t>Grave</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>Caso grave</t>
-  </si>
-  <si>
-    <t>LEVE</t>
-  </si>
-  <si>
-    <t>Leve</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Activo Repetido</t>
-  </si>
-  <si>
     <t>X</t>
   </si>
   <si>
-    <t>Sin Codigo</t>
+    <t>---</t>
   </si>
   <si>
     <t>S</t>
@@ -495,10 +474,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -517,170 +496,146 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="G2">
+      <c r="F3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="C9" t="s">
         <v>27</v>
       </c>
-      <c r="F6" t="s">
+      <c r="D9" t="s">
         <v>28</v>
       </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9">
+      <c r="F9">
         <v>1</v>
       </c>
     </row>

</xml_diff>